<commit_message>
Cambios varios /03/- 2-lu 11:49 PM
</commit_message>
<xml_diff>
--- a/docs/shm_diagrama_despliegue.xlsx
+++ b/docs/shm_diagrama_despliegue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SAN_PABLO\02_HHMM\Desarrollo\ADG_SHM\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C63CFDB-85CB-4C68-BFEA-D6842FA7C087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77DF94F6-EF62-4D4A-BB8A-2FFABF75F2FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{86EF7CFC-75BA-4FD8-A433-F01FE68532FB}"/>
   </bookViews>
@@ -282,11 +282,11 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -692,8 +692,8 @@
       </c>
     </row>
     <row r="43" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="13"/>
-      <c r="C43" s="13"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="14"/>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
@@ -749,7 +749,7 @@
       <c r="H45" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I45" s="14" t="s">
+      <c r="I45" s="13" t="s">
         <v>34</v>
       </c>
       <c r="J45" s="6"/>
@@ -772,7 +772,7 @@
       <c r="H46" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I46" s="14" t="s">
+      <c r="I46" s="13" t="s">
         <v>35</v>
       </c>
       <c r="J46" s="6"/>
@@ -795,7 +795,7 @@
       <c r="H47" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I47" s="14" t="s">
+      <c r="I47" s="13" t="s">
         <v>36</v>
       </c>
       <c r="J47" s="6"/>
@@ -818,7 +818,7 @@
       <c r="H48" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I48" s="14" t="s">
+      <c r="I48" s="13" t="s">
         <v>37</v>
       </c>
       <c r="J48" s="6"/>
@@ -908,7 +908,7 @@
       <c r="H52" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I52" s="14" t="s">
+      <c r="I52" s="13" t="s">
         <v>38</v>
       </c>
       <c r="J52" s="6"/>

</xml_diff>

<commit_message>
Cambios varios /03/- 2-ma 12:07 AM
</commit_message>
<xml_diff>
--- a/docs/shm_diagrama_despliegue.xlsx
+++ b/docs/shm_diagrama_despliegue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SAN_PABLO\02_HHMM\Desarrollo\ADG_SHM\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77DF94F6-EF62-4D4A-BB8A-2FFABF75F2FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{790ECF32-5FBE-49F1-AC5C-0C4853573167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{86EF7CFC-75BA-4FD8-A433-F01FE68532FB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="40">
   <si>
     <t>Componentes</t>
   </si>
@@ -156,6 +156,9 @@
   </si>
   <si>
     <t>whm.notificaciones@sanpablo.com.pe</t>
+  </si>
+  <si>
+    <t>ssss</t>
   </si>
 </sst>
 </file>
@@ -254,7 +257,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -287,6 +290,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -913,6 +919,11 @@
       </c>
       <c r="J52" s="6"/>
     </row>
+    <row r="54" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C54" s="15" t="s">
+        <v>39</v>
+      </c>
+    </row>
     <row r="55" spans="2:10" x14ac:dyDescent="0.25">
       <c r="G55" s="11"/>
     </row>

</xml_diff>

<commit_message>
Cambios varios /04/- 0-do 11:22 PM
</commit_message>
<xml_diff>
--- a/docs/shm_diagrama_despliegue.xlsx
+++ b/docs/shm_diagrama_despliegue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SAN_PABLO\02_HHMM\Desarrollo\ADG_SHM\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{790ECF32-5FBE-49F1-AC5C-0C4853573167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{580BBFDD-5F1E-4ACA-B71D-C852556A9422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{86EF7CFC-75BA-4FD8-A433-F01FE68532FB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
   <si>
     <t>Componentes</t>
   </si>
@@ -156,9 +156,6 @@
   </si>
   <si>
     <t>whm.notificaciones@sanpablo.com.pe</t>
-  </si>
-  <si>
-    <t>ssss</t>
   </si>
 </sst>
 </file>
@@ -288,11 +285,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -698,8 +695,8 @@
       </c>
     </row>
     <row r="43" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
+      <c r="B43" s="15"/>
+      <c r="C43" s="15"/>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
@@ -750,7 +747,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
       <c r="G45" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H45" s="1" t="s">
         <v>12</v>
@@ -773,7 +770,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
       <c r="G46" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H46" s="1" t="s">
         <v>12</v>
@@ -920,9 +917,7 @@
       <c r="J52" s="6"/>
     </row>
     <row r="54" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="C54" s="15" t="s">
-        <v>39</v>
-      </c>
+      <c r="C54" s="14"/>
     </row>
     <row r="55" spans="2:10" x14ac:dyDescent="0.25">
       <c r="G55" s="11"/>

</xml_diff>

<commit_message>
Cambios varios /04/- 0-lu 11:44 PM
</commit_message>
<xml_diff>
--- a/docs/shm_diagrama_despliegue.xlsx
+++ b/docs/shm_diagrama_despliegue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SAN_PABLO\02_HHMM\Desarrollo\ADG_SHM\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{580BBFDD-5F1E-4ACA-B71D-C852556A9422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3985FFD9-C28A-42EA-893D-978F9EA174BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{86EF7CFC-75BA-4FD8-A433-F01FE68532FB}"/>
   </bookViews>
@@ -162,7 +162,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -211,6 +211,15 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -254,7 +263,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -290,6 +299,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -775,7 +787,7 @@
       <c r="H46" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I46" s="13" t="s">
+      <c r="I46" s="16" t="s">
         <v>35</v>
       </c>
       <c r="J46" s="6"/>

</xml_diff>